<commit_message>
Final version for submission. Working
</commit_message>
<xml_diff>
--- a/Data/Output/Out_Classified_Complaints.xlsx
+++ b/Data/Output/Out_Classified_Complaints.xlsx
@@ -40,7 +40,7 @@
     <x:t>Burst pipe near my house</x:t>
   </x:si>
   <x:si>
-    <x:t>0001-01-01</x:t>
+    <x:t>2025-09-01</x:t>
   </x:si>
   <x:si>
     <x:t>Water</x:t>
@@ -55,6 +55,9 @@
     <x:t>Load shedding not on schedule</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-03</x:t>
+  </x:si>
+  <x:si>
     <x:t>Electricity</x:t>
   </x:si>
   <x:si>
@@ -67,6 +70,9 @@
     <x:t>Bin not collected this week</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-27</x:t>
+  </x:si>
+  <x:si>
     <x:t>Refuse</x:t>
   </x:si>
   <x:si>
@@ -79,6 +85,9 @@
     <x:t>Street light not working</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-20</x:t>
+  </x:si>
+  <x:si>
     <x:t>Other</x:t>
   </x:si>
   <x:si>
@@ -91,6 +100,9 @@
     <x:t>No water supply since yesterday</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-05</x:t>
+  </x:si>
+  <x:si>
     <x:t>C006</x:t>
   </x:si>
   <x:si>
@@ -100,75 +112,126 @@
     <x:t>Transformer exploded in my street</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-25</x:t>
+  </x:si>
+  <x:si>
     <x:t>C007</x:t>
   </x:si>
   <x:si>
     <x:t>Rubbish piling up on street corner</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-10</x:t>
+  </x:si>
+  <x:si>
     <x:t>C008</x:t>
   </x:si>
   <x:si>
     <x:t>Potholes on main road</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-30</x:t>
+  </x:si>
+  <x:si>
     <x:t>C009</x:t>
   </x:si>
   <x:si>
     <x:t>Low water pressure in my area</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-07</x:t>
+  </x:si>
+  <x:si>
     <x:t>C010</x:t>
   </x:si>
   <x:si>
     <x:t>No power for 3 days</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-09</x:t>
+  </x:si>
+  <x:si>
     <x:t>C011</x:t>
   </x:si>
   <x:si>
     <x:t>Refuse truck missed our block</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-02</x:t>
+  </x:si>
+  <x:si>
     <x:t>C012</x:t>
   </x:si>
   <x:si>
     <x:t>Illegal dumping near park</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-22</x:t>
+  </x:si>
+  <x:si>
     <x:t>C013</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-28</x:t>
+  </x:si>
+  <x:si>
     <x:t>C014</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-11</x:t>
+  </x:si>
+  <x:si>
     <x:t>C015</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-04</x:t>
+  </x:si>
+  <x:si>
     <x:t>C016</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-26</x:t>
+  </x:si>
+  <x:si>
     <x:t>C017</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-08</x:t>
+  </x:si>
+  <x:si>
     <x:t>C018</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-24</x:t>
+  </x:si>
+  <x:si>
     <x:t>C019</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-06</x:t>
+  </x:si>
+  <x:si>
     <x:t>C020</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-29</x:t>
+  </x:si>
+  <x:si>
     <x:t>C021</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-09-12</x:t>
+  </x:si>
+  <x:si>
     <x:t>C022</x:t>
   </x:si>
   <x:si>
     <x:t>C023</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-23</x:t>
+  </x:si>
+  <x:si>
     <x:t>C024</x:t>
   </x:si>
   <x:si>
@@ -190,6 +253,9 @@
     <x:t>C030</x:t>
   </x:si>
   <x:si>
+    <x:t>2025-08-21</x:t>
+  </x:si>
+  <x:si>
     <x:t>C031</x:t>
   </x:si>
   <x:si>
@@ -259,6 +325,9 @@
     <x:t>Burst pipe causing flooding in the street near my house.</x:t>
   </x:si>
   <x:si>
+    <x:t>2024-03-15</x:t>
+  </x:si>
+  <x:si>
     <x:t>CMP-1002</x:t>
   </x:si>
   <x:si>
@@ -268,6 +337,9 @@
     <x:t>No power since last night due to transformer explosion.</x:t>
   </x:si>
   <x:si>
+    <x:t>2024-03-16</x:t>
+  </x:si>
+  <x:si>
     <x:t>CMP-1003</x:t>
   </x:si>
   <x:si>
@@ -277,6 +349,9 @@
     <x:t>Bin not collected for two weeks and rubbish piling up.</x:t>
   </x:si>
   <x:si>
+    <x:t>2024-03-17</x:t>
+  </x:si>
+  <x:si>
     <x:t>CMP-1004</x:t>
   </x:si>
   <x:si>
@@ -286,6 +361,9 @@
     <x:t>There are potholes on the main road causing traffic issues.</x:t>
   </x:si>
   <x:si>
+    <x:t>2024-03-18</x:t>
+  </x:si>
+  <x:si>
     <x:t>CMP-1005</x:t>
   </x:si>
   <x:si>
@@ -293,6 +371,9 @@
   </x:si>
   <x:si>
     <x:t>Low water pressure in the area; cannot use shower or washing machine properly.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2024-03-19</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -691,58 +772,58 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
         <x:v>9</x:v>
@@ -750,67 +831,67 @@
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
       <x:c r="A8" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
         <x:v>9</x:v>
@@ -818,58 +899,58 @@
     </x:row>
     <x:row r="11" spans="1:5">
       <x:c r="A11" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:5">
       <x:c r="A12" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:5">
       <x:c r="A13" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:5">
       <x:c r="A14" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>6</x:v>
@@ -878,7 +959,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
         <x:v>9</x:v>
@@ -886,67 +967,67 @@
     </x:row>
     <x:row r="15" spans="1:5">
       <x:c r="A15" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:5">
       <x:c r="A16" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:5">
       <x:c r="A17" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:5">
       <x:c r="A18" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
         <x:v>9</x:v>
@@ -954,67 +1035,67 @@
     </x:row>
     <x:row r="19" spans="1:5">
       <x:c r="A19" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:5">
       <x:c r="A20" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:5">
       <x:c r="A21" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:5">
       <x:c r="A22" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
         <x:v>9</x:v>
@@ -1022,67 +1103,67 @@
     </x:row>
     <x:row r="23" spans="1:5">
       <x:c r="A23" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:5">
       <x:c r="A24" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:5">
       <x:c r="A25" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:5">
       <x:c r="A26" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
         <x:v>9</x:v>
@@ -1090,7 +1171,7 @@
     </x:row>
     <x:row r="27" spans="1:5">
       <x:c r="A27" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>11</x:v>
@@ -1099,58 +1180,58 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:5">
       <x:c r="A28" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C28" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:5">
       <x:c r="A29" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:5">
       <x:c r="A30" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C30" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
         <x:v>9</x:v>
@@ -1158,67 +1239,67 @@
     </x:row>
     <x:row r="31" spans="1:5">
       <x:c r="A31" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C31" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:5">
       <x:c r="A32" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:5">
       <x:c r="A33" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C33" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:5">
       <x:c r="A34" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C34" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
         <x:v>9</x:v>
@@ -1226,58 +1307,58 @@
     </x:row>
     <x:row r="35" spans="1:5">
       <x:c r="A35" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:5">
       <x:c r="A36" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C36" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:5">
       <x:c r="A37" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C37" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:5">
       <x:c r="A38" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>6</x:v>
@@ -1286,7 +1367,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E38" s="0" t="s">
         <x:v>9</x:v>
@@ -1294,64 +1375,64 @@
     </x:row>
     <x:row r="39" spans="1:5">
       <x:c r="A39" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C39" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:5">
       <x:c r="A40" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C40" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E40" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:5">
       <x:c r="A41" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C41" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E41" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:5">
       <x:c r="A42" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C42" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
         <x:v>8</x:v>
@@ -1362,67 +1443,67 @@
     </x:row>
     <x:row r="43" spans="1:5">
       <x:c r="A43" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C43" s="0" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E43" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:5">
       <x:c r="A44" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C44" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E44" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:5">
       <x:c r="A45" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C45" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E45" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:5">
       <x:c r="A46" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C46" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E46" s="0" t="s">
         <x:v>9</x:v>
@@ -1430,58 +1511,58 @@
     </x:row>
     <x:row r="47" spans="1:5">
       <x:c r="A47" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C47" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E47" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:5">
       <x:c r="A48" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C48" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E48" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:5">
       <x:c r="A49" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C49" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E49" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:5">
       <x:c r="A50" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>6</x:v>
@@ -1490,7 +1571,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E50" s="0" t="s">
         <x:v>9</x:v>
@@ -1498,33 +1579,33 @@
     </x:row>
     <x:row r="51" spans="1:5">
       <x:c r="A51" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="C51" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E51" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:5">
       <x:c r="A52" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C52" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D52" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E52" s="0" t="s">
         <x:v>9</x:v>
@@ -1532,67 +1613,67 @@
     </x:row>
     <x:row r="53" spans="1:5">
       <x:c r="A53" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C53" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D53" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E53" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:5">
       <x:c r="A54" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C54" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E54" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:5">
       <x:c r="A55" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C55" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E55" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:5">
       <x:c r="A56" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C56" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E56" s="0" t="s">
         <x:v>9</x:v>

</xml_diff>